<commit_message>
made changes in the button content, prompt
</commit_message>
<xml_diff>
--- a/llm_stats/token_usage.xlsx
+++ b/llm_stats/token_usage.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX33"/>
+  <dimension ref="A1:AX35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -8325,6 +8325,490 @@
       </c>
       <c r="AX33" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>11e93a4e-a4a7-4823-9fdc-dd5e102c9699</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-03-17 10:10:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>399</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Evaluate Division</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/evaluate-division/description/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>f5a6ffb323aa4bf37798407ac922df77aeb4487c2c69de185e5bc8d4f851e44d</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>You are an expert technical writer creating a high-quality LeetCode solution post. Problem Details: Number: 399 Name: Evaluate Division Difficulty: medium Link: https://leetcode.com/problems/evaluate-division/description/ Python Solution: from collections import defaultdict cl...</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are an expert technical writer creating a high-quality LeetCode solution post.
+Problem Details:
+Number: 399
+Name: Evaluate Division
+Difficulty: medium
+Link: https://leetcode.com/problems/evaluate-division/description/
+Python Solution:
+from collections import defaultdict
+class Solution:
+    def calcEquation(self, equations: List[List[str]], values: List[float], queries: List[List[str]]) -&gt; List[float]:
+        mapping = defaultdict(list)
+        for (a,b),c in zip(equations,values):
+            mapping[a].append([b,c])
+            mapping[b].append([a,1/c])
+        def dfs(curr,target,visited):
+            if curr == target:
+                return 1.0
+            visited.add(curr)
+            for i,j in mapping[curr]:
+                if i not in visited:
+                    res = dfs(i,target,visited)
+                    if res != -1:
+                        return res*j
+            return -1
+        result = []
+        for i,j in queries:
+            if i not in mapping.keys() or j not in mapping.keys():
+                result.append(-1.0)
+            else:
+                result.append(dfs(i,j,set()))
+        return result
+Instructions:
+1. Generate a strong, descriptive, professional Title.
+- The title MUST mention:
+    - The core technique used
+    - The time complexity (Big-O notation)
+- The explanation must match the provided language
+- IMPORTANT: The title text (after "Title: ") must be 75 characters or fewer.
+- IMPORTANT: The title MUST be a fully complete, grammatically whole phrase — never cut off mid-word or mid-sentence. Plan the title length upfront so that the entire title fits within 75 characters naturally. If a draft title is too long, shorten it by simplifying words, not by truncating.
+2. Generate markdown using exactly these sections and no additional top-level sections:
+Title: &lt;single line title, max 75 characters&gt;
+## Intuition
+## Approach
+## Time Complexity
+## Space Complexity
+3. Do NOT include any code block and do NOT add a ## Code section.
+4. Keep the response concise, technical, and ready for markdown publishing.
+</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>2087</v>
+      </c>
+      <c r="O34" t="n">
+        <v>58</v>
+      </c>
+      <c r="P34" t="n">
+        <v>910</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>28</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>cfd455fc6745267dd8b187dafb79223ecdaf3c589d49fc74d75fa0b689e55723</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>from collections import defaultdict
+class Solution:
+    def calcEquation(self, equations: List[List[str]], values: List[float], queries: List[List[str]]) -&gt; List[float]:
+        mapping = defaultdict(list)
+        for (a,b),c in zip(equations,values):
+            mapping[a].append([b,c])
+            mapping[b].append([a,1/c])
+        def dfs(curr,target,visited):
+            if curr == target:
+                return 1.0
+            visited.add(curr)
+            for i,j in mapping[curr]:
+                if i not in visited:
+                    res = dfs(i,target,visited)
+                    if res != -1:
+                        return res*j
+            return -1
+        result = []
+        for i,j in queries:
+            if i not in mapping.keys() or j not in mapping.keys():
+                result.append(-1.0)
+            else:
+                result.append(dfs(i,j,set()))
+        return result</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>580</v>
+      </c>
+      <c r="U34" t="n">
+        <v>375</v>
+      </c>
+      <c r="V34" t="n">
+        <v>955</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.6466</v>
+      </c>
+      <c r="X34" t="n">
+        <v>91889.02</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>5629.65</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>25859.3</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>60298.05</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>6.2191</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>1697</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>19</v>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>Title: Depth-First Search based Graph Traversal with Floyd-Warshall's Distance Algorithm Optimization (Medium)
+## Intuition
+The problem can be approached using graph theory. We represent the given equations as a weighted graph where each node corresponds to a variable, and the edges are connected by the coefficients of their respective equations. The weights of these edges are the values associated with the equations.
+## Approach
+Our solution initializes a dictionary `mapping` that stores pairs of variables (nodes) and their corresponding weighted edges. After that, we implement a depth-first search (DFS) function to traverse the graph and find the product of the coefficients between two nodes if they are connected. If there is no direct connection, we return -1.
+In addition, we optimize DFS using Floyd-Warshall's algorithm to calculate the shortest distances between all pairs of nodes in the graph. This optimization allows us to perform multiple queries more efficiently without recomputing the distances for each query.
+## Time Complexity
+The time complexity of our solution is O(N^3), where N is the number of variables, due to the use of Floyd-Warshall's algorithm for optimizing the DFS function. This is because we perform three nested loops to calculate shortest paths between all pairs of nodes in the graph.
+## Space Complexity
+The space complexity of our solution is O(N^2) due to the use of the `mapping` dictionary and an additional space requirement for storing shortest distances during the Floyd-Warshall algorithm. This is because each node is connected to other nodes, and we also need to store intermediate calculations during the Floyd-Warshall algorithm.</t>
+        </is>
+      </c>
+      <c r="AL34" t="n">
+        <v>2680</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>54</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4f20a172-adb3-4156-9d39-35fe558bfbee</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-03-17 10:17:43</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>997</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Find the Town Judge</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/find-the-town-judge/description/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>c7ac6599fefeeb4bca3a507875558c646b43c102955296b3134418b388efb013</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>You are an expert technical writer creating a high-quality LeetCode solution post. Problem Details: Number: 997 Name: Find the Town Judge Difficulty: easy Link: https://leetcode.com/problems/find-the-town-judge/description/ Python Solution: from collections import defaultdict ...</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are an expert technical writer creating a high-quality LeetCode solution post.
+Problem Details:
+Number: 997
+Name: Find the Town Judge
+Difficulty: easy
+Link: https://leetcode.com/problems/find-the-town-judge/description/
+Python Solution:
+from collections import defaultdict
+class Solution:
+    def findJudge(self, n: int, trust: List[List[int]]) -&gt; int:
+        indegree = [0]*(n+1)
+        outdegree = [0]*(n+1)
+        for a,b in trust:
+            outdegree[a] += 1
+            indegree[b] += 1
+        for i in range(1,n+1):
+            if indegree[i] == n-1 and outdegree[i] == 0:
+                return i
+        return -1
+Instructions:
+1. Generate a strong, descriptive, professional Title.
+- The title MUST mention:
+    - The core technique used
+    - The time complexity (Big-O notation)
+- The explanation must match the provided language
+- IMPORTANT: The title text (after "Title: ") must be 75 characters or fewer.
+- IMPORTANT: The title MUST be a fully complete, grammatically whole phrase — never cut off mid-word or mid-sentence. Plan the title length upfront so that the entire title fits within 75 characters naturally. If a draft title is too long, shorten it by simplifying words, not by truncating.
+2. Generate markdown using exactly these sections and no additional top-level sections:
+Title: &lt;single line title, max 75 characters&gt;
+## Intuition
+## Approach
+## Time Complexity
+## Space Complexity
+3. Do NOT include any code block and do NOT add a ## Code section.
+4. Keep the response concise, technical, and ready for markdown publishing.
+</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>1597</v>
+      </c>
+      <c r="O35" t="n">
+        <v>46</v>
+      </c>
+      <c r="P35" t="n">
+        <v>418</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>16</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>7fca0c714e7536e1c77f8ad567dfcbd5f70b1a909434e3155a9868a097e90a67</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>from collections import defaultdict
+class Solution:
+    def findJudge(self, n: int, trust: List[List[int]]) -&gt; int:
+        indegree = [0]*(n+1)
+        outdegree = [0]*(n+1)
+        for a,b in trust:
+            outdegree[a] += 1
+            indegree[b] += 1
+        for i in range(1,n+1):
+            if indegree[i] == n-1 and outdegree[i] == 0:
+                return i
+        return -1</t>
+        </is>
+      </c>
+      <c r="T35" t="n">
+        <v>467</v>
+      </c>
+      <c r="U35" t="n">
+        <v>360</v>
+      </c>
+      <c r="V35" t="n">
+        <v>827</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0.7709</v>
+      </c>
+      <c r="X35" t="n">
+        <v>83826.21000000001</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>5630.87</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>19822.94</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>58281.38</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>6.1769</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>1479</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>20</v>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>Title: Graph-based Technique with Linear Time Complexity (O(n)) for Find Town Judge Problem on LeetCode
+## Intuition
+The solution is based on analyzing the given trust relationships within a town. A judge in the town is a person who everyone else in the town does not trust, but he trusts no one. In this problem, we keep count of incoming (trusting) and outgoing (being trusted) connections for each resident using adjacency lists.
+## Approach
+1. Initialize an array `indegree` to keep track of the inbound connections for each resident and another array `outdegree` to keep track of the outbound connections.
+2. Iterate through the trust relationships, incrementing the corresponding outdegree and indegree values.
+3. Check each resident's indegree (incoming connections) and outdegree (outgoing connections). If a resident has an indegree of `n-1` (everyone else in the town does not trust them) and an outdegree of 0, they are the judge.
+4. If no resident matches these conditions, return -1 as there is no town judge.
+## Time Complexity
+The time complexity of this solution is O(n), where n represents the number of residents in the town. This is due to the linear operations on the arrays to initialize and iterate through the trust relationships.
+## Space Complexity
+The space complexity for this solution is O(n) since we are using two arrays (`indegree` and `outdegree`) of size n, along with the input arrays for the number of residents and trust relationships.</t>
+        </is>
+      </c>
+      <c r="AL35" t="n">
+        <v>1977</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX35" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8358,7 +8842,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -8368,7 +8852,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -8398,7 +8882,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.94</v>
+        <v>5.95</v>
       </c>
     </row>
     <row r="7">
@@ -8408,7 +8892,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>124413.61</v>
+        <v>122263.26</v>
       </c>
     </row>
     <row r="8">
@@ -8418,7 +8902,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>98.44</v>
+        <v>98.53</v>
       </c>
     </row>
     <row r="9">
@@ -8428,7 +8912,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>98.44</v>
+        <v>98.53</v>
       </c>
     </row>
   </sheetData>
@@ -8442,7 +8926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9390,22 +9874,96 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>c7ac6599fefeeb4bca3a507875558c646b43c102955296b3134418b388efb013</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>100</v>
+      </c>
+      <c r="G26" t="n">
+        <v>100</v>
+      </c>
+      <c r="H26" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.7709</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>f5a6ffb323aa4bf37798407ac922df77aeb4487c2c69de185e5bc8d4f851e44d</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>100</v>
+      </c>
+      <c r="G27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H27" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.6466</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>mistral:latest</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>f7015d8f6a2ee4ab28fb4702bade95ce459f3f16948c137835f4ba4cab21668b</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="n">
-        <v>100</v>
-      </c>
-      <c r="G26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H26" t="n">
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H28" t="n">
         <v>6.05</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I28" t="n">
         <v>0.8605</v>
       </c>
     </row>
@@ -9453,39 +10011,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>mistral:latest</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>17</v>
       </c>
       <c r="C2" t="n">
-        <v>5.8</v>
+        <v>6.11</v>
       </c>
       <c r="D2" t="n">
-        <v>126706.12</v>
+        <v>117820.39</v>
       </c>
       <c r="E2" t="n">
-        <v>99.02</v>
+        <v>98.04000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mistral:latest</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="D3" t="n">
-        <v>121815.43</v>
+        <v>126706.12</v>
       </c>
       <c r="E3" t="n">
-        <v>97.78</v>
+        <v>99.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>